<commit_message>
Fix: Solucionar cierre inmediato de ejecutar.bat con CRLF, diagnostico integrado, validacion estricta y soporte para busquedas individuales con comas
</commit_message>
<xml_diff>
--- a/reporte_supermercados.xlsx
+++ b/reporte_supermercados.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="100">
   <si>
     <t>🛒 REPORTE RPA: COMPARADOR DE PRECIOS Y CANASTA INTELIGENTE</t>
   </si>
@@ -35,37 +35,49 @@
     <t>💸 AHORRO MÁXIMO</t>
   </si>
   <si>
+    <t>COTO</t>
+  </si>
+  <si>
+    <t>📊 EVALUACIÓN COMPARATIVA: COSTO TOTAL DE LA CANASTA COMPLETA</t>
+  </si>
+  <si>
+    <t>Supermercado</t>
+  </si>
+  <si>
+    <t>Costo Canasta Total</t>
+  </si>
+  <si>
+    <t>Artículos Disponibles</t>
+  </si>
+  <si>
+    <t>Artículos con Problema</t>
+  </si>
+  <si>
+    <t>Precios Más Bajos Ganados</t>
+  </si>
+  <si>
+    <t>Diferencia vs Mejor</t>
+  </si>
+  <si>
+    <t>Estado / Recomendación</t>
+  </si>
+  <si>
     <t>Carrefour</t>
   </si>
   <si>
-    <t>📊 EVALUACIÓN COMPARATIVA: COSTO TOTAL DE LA CANASTA COMPLETA</t>
-  </si>
-  <si>
-    <t>Supermercado</t>
-  </si>
-  <si>
-    <t>Costo Canasta Total</t>
-  </si>
-  <si>
-    <t>Artículos Disponibles</t>
-  </si>
-  <si>
-    <t>Artículos con Problema</t>
-  </si>
-  <si>
-    <t>Precios Más Bajos Ganados</t>
-  </si>
-  <si>
-    <t>Diferencia vs Mejor</t>
-  </si>
-  <si>
-    <t>Estado / Recomendación</t>
-  </si>
-  <si>
-    <t>5 de 5</t>
-  </si>
-  <si>
-    <t>2 productos</t>
+    <t>2 de 2</t>
+  </si>
+  <si>
+    <t>0 productos</t>
+  </si>
+  <si>
+    <t>+$31,00</t>
+  </si>
+  <si>
+    <t>Más costoso</t>
+  </si>
+  <si>
+    <t>1 productos</t>
   </si>
   <si>
     <t>Mejor opción</t>
@@ -74,22 +86,10 @@
     <t>🏆 RECOMENDADO</t>
   </si>
   <si>
-    <t>COTO</t>
-  </si>
-  <si>
-    <t>1 productos</t>
-  </si>
-  <si>
-    <t>+$65,85</t>
-  </si>
-  <si>
-    <t>Más costoso</t>
-  </si>
-  <si>
     <t>Día %</t>
   </si>
   <si>
-    <t>+$1.507,00</t>
+    <t>+$739,50</t>
   </si>
   <si>
     <t>🛒 PRODUCTO GANADOR POR ARTÍCULO (MEJOR PRECIO)</t>
@@ -116,81 +116,42 @@
     <t>Enlace Directo</t>
   </si>
   <si>
-    <t>YERBA</t>
+    <t>LECHE</t>
+  </si>
+  <si>
+    <t>🏆 COTO</t>
+  </si>
+  <si>
+    <t>Leche descremada larga vida con proteína LAS TRES NIÑAS 1L</t>
+  </si>
+  <si>
+    <t>Día % ($3.500)</t>
+  </si>
+  <si>
+    <t>-$1.250</t>
+  </si>
+  <si>
+    <t>🔗 Ver en Tienda</t>
+  </si>
+  <si>
+    <t>ARROZ</t>
   </si>
   <si>
     <t>🏆 Día %</t>
   </si>
   <si>
-    <t>Yerba Mate Mañanita 4 Flex 1 Kg.</t>
-  </si>
-  <si>
-    <t>COTO ($5.370)</t>
-  </si>
-  <si>
-    <t>-$1.580</t>
-  </si>
-  <si>
-    <t>🔗 Ver en Tienda</t>
-  </si>
-  <si>
-    <t>LECHE</t>
-  </si>
-  <si>
-    <t>🏆 COTO</t>
-  </si>
-  <si>
-    <t>Leche descremada larga vida con proteína LAS TRES NIÑAS 1L</t>
-  </si>
-  <si>
-    <t>Día % ($3.335)</t>
-  </si>
-  <si>
-    <t>-$1.085</t>
-  </si>
-  <si>
-    <t>ARROZ</t>
-  </si>
-  <si>
-    <t>Arroz Largo Fino Ala 1 Kg.</t>
-  </si>
-  <si>
-    <t>Carrefour ($1.940)</t>
-  </si>
-  <si>
-    <t>-$450</t>
-  </si>
-  <si>
-    <t>FIDEOS</t>
-  </si>
-  <si>
-    <t>🏆 Carrefour</t>
-  </si>
-  <si>
-    <t>Fideos tallarin N5 Lucchetti 500 g.</t>
-  </si>
-  <si>
-    <t>Día % ($1.900)</t>
-  </si>
-  <si>
-    <t>-$765</t>
-  </si>
-  <si>
-    <t>ACEITE</t>
-  </si>
-  <si>
-    <t>Aceite de girasol alto omega Carrefour Classic pet 1.5 lts</t>
-  </si>
-  <si>
-    <t>Día % ($7.800)</t>
-  </si>
-  <si>
-    <t>-$2.395</t>
+    <t>Arroz Parboil Molinos Ala 1 Kg.</t>
+  </si>
+  <si>
+    <t>COTO ($1.999)</t>
+  </si>
+  <si>
+    <t>-$510,5</t>
   </si>
   <si>
     <t xml:space="preserve">💡 CONCLUSIÓN Y ESTRATEGIA RECOMENDADA POR EL BOT RPA:
-1. Si realizás toda la compra mensual en un único lugar: El supermercado más conveniente es Carrefour con un costo de $16.808,00.
-2. Si realizás una compra combinada (comprando cada producto en su supermercado ganador): Pagás solo $14.070,00, ahorrando un total de $4.245,00.
+1. Si realizás toda la compra mensual en un único lugar: El supermercado más conveniente es COTO con un costo de $4.249,00.
+2. Si realizás una compra combinada (comprando cada producto en su supermercado ganador): Pagás solo $3.738,50, ahorrando un total de $1.250,00.
 3. Podés verificar el detalle de stock y sustituciones rechazadas en la pestaña "⚠️ Disponibilidad y Stock".</t>
   </si>
   <si>
@@ -209,19 +170,10 @@
     <t>Ahorro Máximo</t>
   </si>
   <si>
-    <t>-$1.580,00</t>
-  </si>
-  <si>
-    <t>-$1.085,00</t>
-  </si>
-  <si>
-    <t>-$450,00</t>
-  </si>
-  <si>
-    <t>-$765,00</t>
-  </si>
-  <si>
-    <t>-$2.395,00</t>
+    <t>-$1.250,00</t>
+  </si>
+  <si>
+    <t>-$510,50</t>
   </si>
   <si>
     <t>TOTAL CANASTA</t>
@@ -230,9 +182,6 @@
     <t>Óptima Combinada</t>
   </si>
   <si>
-    <t>-$4.245,00</t>
-  </si>
-  <si>
     <t>📊 RANKING GENERAL: TODOS LOS PRODUCTOS DE MENOR A MAYOR PRECIO</t>
   </si>
   <si>
@@ -269,117 +218,42 @@
     <t>🥈 2° Puesto</t>
   </si>
   <si>
-    <t>Fideos Spaghetti N° 7 LUCCHETTI 500g</t>
+    <t>Arroz largo fino Molinos Ala 1 kg.</t>
   </si>
   <si>
     <t>🥉 3° Puesto</t>
   </si>
   <si>
+    <t>Arroz Largo Fino LUCCHETTI 1kg</t>
+  </si>
+  <si>
     <t>#4</t>
   </si>
   <si>
-    <t>Arroz Largo Fino LUCCHETTI 1kg</t>
-  </si>
-  <si>
     <t>#5</t>
   </si>
   <si>
-    <t>Fideos tirabuzon integral n28 Matarazzo 500 Gr.</t>
+    <t>Leche Protein La Serenisima 1L</t>
   </si>
   <si>
     <t>#6</t>
   </si>
   <si>
-    <t>Arroz largo fino Molinos Ala 1 kg.</t>
+    <t>Danette Postre Sabor Dulce De Leche Pack X2 95 Gr.</t>
   </si>
   <si>
     <t>#7</t>
   </si>
   <si>
-    <t>LECHE SERENISIMA</t>
-  </si>
-  <si>
-    <t>Leche Multidefensas 3% LA SERENISIMA Sachet 1l</t>
+    <t>COCA COLA, 2.25L</t>
+  </si>
+  <si>
+    <t>Gaseosa Coca-Cola Zero 2.25 Lt.</t>
   </si>
   <si>
     <t>🔎 Individual</t>
   </si>
   <si>
-    <t>#8</t>
-  </si>
-  <si>
-    <t>#9</t>
-  </si>
-  <si>
-    <t>Leche fresca Zero Lactosa La Serenisima 1 Lt.</t>
-  </si>
-  <si>
-    <t>#10</t>
-  </si>
-  <si>
-    <t>COCA COLA</t>
-  </si>
-  <si>
-    <t>Gaseosa Coca-Cola Sabor Original 600 Ml.</t>
-  </si>
-  <si>
-    <t>#11</t>
-  </si>
-  <si>
-    <t>Leche Protein La Serenisima 1L</t>
-  </si>
-  <si>
-    <t>#12</t>
-  </si>
-  <si>
-    <t>#13</t>
-  </si>
-  <si>
-    <t>Leche Infantil Nutrilon Profutura Etapa 1 Brick 200 Ml.</t>
-  </si>
-  <si>
-    <t>#14</t>
-  </si>
-  <si>
-    <t>#15</t>
-  </si>
-  <si>
-    <t>Gaseosa cola Coca Cola Zero 2,25 lts</t>
-  </si>
-  <si>
-    <t>#16</t>
-  </si>
-  <si>
-    <t>Gaseosa Coca-Cola Sabor Original 2,25 Lt</t>
-  </si>
-  <si>
-    <t>#17</t>
-  </si>
-  <si>
-    <t>Yerba mate Playadito suave con palo 1 kg.</t>
-  </si>
-  <si>
-    <t>#18</t>
-  </si>
-  <si>
-    <t>Yerba Mate 4 Flex Mañanita Paq 1 Kgm</t>
-  </si>
-  <si>
-    <t>#19</t>
-  </si>
-  <si>
-    <t>#20</t>
-  </si>
-  <si>
-    <t>Aceite Girasol CAÑUELAS Botella 1.5 L</t>
-  </si>
-  <si>
-    <t>#21</t>
-  </si>
-  <si>
-    <t>Aceite Oliva Extra Virgen La Toscana 250 Ml.</t>
-  </si>
-  <si>
     <t>🔎 HISTORIAL DE BÚSQUEDAS INDIVIDUALES Y VALIDACIONES EN VIVO</t>
   </si>
   <si>
@@ -395,43 +269,31 @@
     <t>Observación Técnica</t>
   </si>
   <si>
-    <t>2026-09-08</t>
-  </si>
-  <si>
-    <t>leche serenisima</t>
+    <t>2026-09-09</t>
+  </si>
+  <si>
+    <t>Coca Cola, 2.25L</t>
+  </si>
+  <si>
+    <t>Gaseosa Coca-Cola Zero 600 ml</t>
+  </si>
+  <si>
+    <t>❌ COINCIDENCIA NO VÁLIDA</t>
+  </si>
+  <si>
+    <t>Presentación incompatible: solicitada 2.25l vs encontrada 600 ml.</t>
+  </si>
+  <si>
+    <t>Gaseosa Zero COCA COLA 1.25l</t>
+  </si>
+  <si>
+    <t>Presentación incompatible: solicitada 2.25l vs encontrada 1.25l.</t>
   </si>
   <si>
     <t xml:space="preserve"> VALIDADA</t>
   </si>
   <si>
     <t>Coincidencia específica validada (marca, categoría y atributos conformes).</t>
-  </si>
-  <si>
-    <t>pomelo Secco</t>
-  </si>
-  <si>
-    <t>Shampoo Dove Nutrición + Tri-Óleos 400 ml</t>
-  </si>
-  <si>
-    <t>❌ COINCIDENCIA NO VÁLIDA</t>
-  </si>
-  <si>
-    <t>Marca requerida "SECCO" no coincide con el producto devuelto ("Shampoo Dove Nutrición + Tri-Óleos 400 ml").</t>
-  </si>
-  <si>
-    <t>Pomelo Rojo . Xkg</t>
-  </si>
-  <si>
-    <t>Marca requerida "SECCO" no coincide con el producto devuelto ("Pomelo Rojo . Xkg").</t>
-  </si>
-  <si>
-    <t>Shampoo Pantene Pro-V Miracles Keratina Repara y Protege Reparador 300 Ml.</t>
-  </si>
-  <si>
-    <t>Marca requerida "SECCO" no coincide con el producto devuelto ("Shampoo Pantene Pro-V Miracles Keratina Repara y Protege Reparador 300 Ml.").</t>
-  </si>
-  <si>
-    <t>coca cola</t>
   </si>
   <si>
     <t>⚠️ REPORTE DE DISPONIBILIDAD: ARTÍCULOS SIN STOCK O RECHAZADOS POR VALIDACIÓN</t>
@@ -515,17 +377,17 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF333333"/>
+    </font>
+    <font>
+      <color rgb="FF666666"/>
+    </font>
+    <font>
+      <color rgb="FF777777"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="276A3C"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF333333"/>
-    </font>
-    <font>
-      <color rgb="FF666666"/>
-    </font>
-    <font>
-      <color rgb="FF777777"/>
     </font>
     <font>
       <b/>
@@ -577,15 +439,15 @@
       <color rgb="FF666666"/>
       <sz val="8"/>
     </font>
-    <font>
-      <color rgb="FF555555"/>
-      <sz val="8"/>
-    </font>
     <font/>
     <font>
       <b/>
       <color rgb="C00000"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="FF555555"/>
+      <sz val="8"/>
     </font>
     <font>
       <b/>
@@ -714,25 +576,25 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -768,7 +630,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -789,14 +651,14 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1149,7 +1011,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H25"/>
+  <dimension ref="B2:H22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1206,15 +1068,15 @@
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="5">
-        <v>16808</v>
+        <v>4249</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="6">
-        <v>14070</v>
+        <v>3738.5</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6">
-        <v>4245</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -1253,36 +1115,36 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="9" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C10" s="10">
-        <v>16808</v>
+        <v>4280</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E10" s="11">
         <v>0</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C11" s="14">
-        <v>16873.85</v>
+        <v>4249</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E11" s="11">
         <v>0</v>
@@ -1301,23 +1163,23 @@
       <c r="B12" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="14">
-        <v>18315</v>
+      <c r="C12" s="10">
+        <v>4988.5</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E12" s="11">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="G12" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="16" t="s">
-        <v>22</v>
+      <c r="H12" s="13" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -1364,8 +1226,8 @@
       <c r="D16" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="10">
-        <v>3790</v>
+      <c r="E16" s="14">
+        <v>2250</v>
       </c>
       <c r="F16" s="20" t="s">
         <v>36</v>
@@ -1387,8 +1249,8 @@
       <c r="D17" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E17" s="10">
-        <v>2250</v>
+      <c r="E17" s="14">
+        <v>1488.5</v>
       </c>
       <c r="F17" s="20" t="s">
         <v>42</v>
@@ -1400,112 +1262,43 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" s="17" t="s">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="E18" s="10">
-        <v>1490</v>
-      </c>
-      <c r="F18" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="G18" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="H18" s="22" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="E19" s="10">
-        <v>1135</v>
-      </c>
-      <c r="F19" s="20" t="s">
-        <v>51</v>
-      </c>
-      <c r="G19" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="H19" s="22" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="C20" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20" s="10">
-        <v>5405</v>
-      </c>
-      <c r="F20" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="G20" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="H20" s="22" t="s">
-        <v>38</v>
-      </c>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="23" t="s">
-        <v>57</v>
-      </c>
+      <c r="B22" s="23"/>
       <c r="C22" s="23"/>
       <c r="D22" s="23"/>
       <c r="E22" s="23"/>
       <c r="F22" s="23"/>
       <c r="G22" s="23"/>
       <c r="H22" s="23"/>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="G23" s="23"/>
-      <c r="H23" s="23"/>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="23"/>
-      <c r="G24" s="23"/>
-      <c r="H24" s="23"/>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="G25" s="23"/>
-      <c r="H25" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1519,14 +1312,11 @@
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B22:H25"/>
+    <mergeCell ref="B19:H22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H16" r:id="rId1"/>
     <hyperlink ref="H17" r:id="rId2"/>
-    <hyperlink ref="H18" r:id="rId3"/>
-    <hyperlink ref="H19" r:id="rId4"/>
-    <hyperlink ref="H20" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1535,7 +1325,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H11"/>
+  <dimension ref="B2:H8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1547,7 +1337,7 @@
   <sheetData>
     <row r="2" ht="34" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -1558,7 +1348,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
@@ -1572,22 +1362,22 @@
         <v>26</v>
       </c>
       <c r="C5" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="26" t="s">
         <v>6</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>19</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>23</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -1595,22 +1385,22 @@
         <v>33</v>
       </c>
       <c r="C6" s="27">
-        <v>5209</v>
-      </c>
-      <c r="D6" s="27">
-        <v>5370</v>
-      </c>
-      <c r="E6" s="10">
-        <v>3790</v>
-      </c>
-      <c r="F6" s="13" t="s">
+        <v>2340</v>
+      </c>
+      <c r="D6" s="14">
+        <v>2250</v>
+      </c>
+      <c r="E6" s="27">
+        <v>3500</v>
+      </c>
+      <c r="F6" s="16" t="s">
         <v>34</v>
       </c>
       <c r="G6" s="28">
-        <v>3790</v>
-      </c>
-      <c r="H6" s="12" t="s">
-        <v>63</v>
+        <v>2250</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -1618,114 +1408,45 @@
         <v>39</v>
       </c>
       <c r="C7" s="27">
-        <v>3119</v>
-      </c>
-      <c r="D7" s="10">
-        <v>2250</v>
-      </c>
-      <c r="E7" s="27">
-        <v>3335</v>
-      </c>
-      <c r="F7" s="13" t="s">
+        <v>1940</v>
+      </c>
+      <c r="D7" s="27">
+        <v>1999</v>
+      </c>
+      <c r="E7" s="14">
+        <v>1488.5</v>
+      </c>
+      <c r="F7" s="16" t="s">
         <v>40</v>
       </c>
       <c r="G7" s="28">
-        <v>2250</v>
-      </c>
-      <c r="H7" s="12" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" s="27">
-        <v>1940</v>
-      </c>
-      <c r="D8" s="27">
-        <v>1498.85</v>
-      </c>
-      <c r="E8" s="10">
-        <v>1490</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="G8" s="28">
-        <v>1490</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="10">
-        <v>1135</v>
-      </c>
-      <c r="D9" s="27">
-        <v>1225</v>
-      </c>
-      <c r="E9" s="27">
-        <v>1900</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="G9" s="28">
-        <v>1135</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="9" t="s">
+        <v>1488.5</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="30">
+        <v>4280</v>
+      </c>
+      <c r="D8" s="14">
+        <v>4249</v>
+      </c>
+      <c r="E8" s="30">
+        <v>4988.5</v>
+      </c>
+      <c r="F8" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="10">
-        <v>5405</v>
-      </c>
-      <c r="D10" s="27">
-        <v>6530</v>
-      </c>
-      <c r="E10" s="27">
-        <v>7800</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="G10" s="28">
-        <v>5405</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="C11" s="10">
-        <v>16808</v>
-      </c>
-      <c r="D11" s="30">
-        <v>16873.85</v>
-      </c>
-      <c r="E11" s="30">
-        <v>18315</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="G11" s="10">
-        <v>14070</v>
-      </c>
-      <c r="H11" s="12" t="s">
-        <v>70</v>
+      <c r="G8" s="14">
+        <v>3738.5</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1740,7 +1461,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H26"/>
+  <dimension ref="B2:H12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1755,7 +1476,7 @@
   <sheetData>
     <row r="2" ht="34" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -1766,7 +1487,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
@@ -1777,508 +1498,186 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="26" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="C5" s="26" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="13" t="s">
-        <v>79</v>
+      <c r="B6" s="16" t="s">
+        <v>62</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="F6" s="28">
-        <v>1135</v>
+        <v>1488.5</v>
       </c>
       <c r="G6" s="32" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="33" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="F7" s="28">
-        <v>1225</v>
+        <v>1940</v>
       </c>
       <c r="G7" s="32" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="H7" s="22" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="33" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="F8" s="28">
-        <v>1490</v>
+        <v>1999</v>
       </c>
       <c r="G8" s="32" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="34" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="F9" s="14">
-        <v>1498.85</v>
+        <v>35</v>
+      </c>
+      <c r="F9" s="10">
+        <v>2250</v>
       </c>
       <c r="G9" s="32" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="34" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="F10" s="14">
-        <v>1900</v>
+        <v>71</v>
+      </c>
+      <c r="F10" s="10">
+        <v>2340</v>
       </c>
       <c r="G10" s="32" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="34" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="F11" s="14">
-        <v>1940</v>
+        <v>73</v>
+      </c>
+      <c r="F11" s="10">
+        <v>3500</v>
       </c>
       <c r="G11" s="32" t="s">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="H11" s="22" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="34" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="F12" s="14">
-        <v>2140</v>
+        <v>76</v>
+      </c>
+      <c r="F12" s="10">
+        <v>5900</v>
       </c>
       <c r="G12" s="32" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="H12" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="34" t="s">
-        <v>95</v>
-      </c>
-      <c r="C13" s="31" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="E13" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" s="14">
-        <v>2250</v>
-      </c>
-      <c r="G13" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H13" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="C14" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>97</v>
-      </c>
-      <c r="F14" s="14">
-        <v>2375</v>
-      </c>
-      <c r="G14" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="H14" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B15" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="C15" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="E15" s="19" t="s">
-        <v>100</v>
-      </c>
-      <c r="F15" s="14">
-        <v>2600</v>
-      </c>
-      <c r="G15" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="H15" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B16" s="34" t="s">
-        <v>101</v>
-      </c>
-      <c r="C16" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="E16" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="F16" s="14">
-        <v>3119</v>
-      </c>
-      <c r="G16" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H16" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B17" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="C17" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="E17" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="F17" s="14">
-        <v>3119</v>
-      </c>
-      <c r="G17" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="H17" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="C18" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>105</v>
-      </c>
-      <c r="F18" s="14">
-        <v>3335</v>
-      </c>
-      <c r="G18" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H18" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="34" t="s">
-        <v>106</v>
-      </c>
-      <c r="C19" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="F19" s="14">
-        <v>3790</v>
-      </c>
-      <c r="G19" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H19" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="C20" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="E20" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="F20" s="14">
-        <v>4425</v>
-      </c>
-      <c r="G20" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="H20" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B21" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="C21" s="31" t="s">
-        <v>19</v>
-      </c>
-      <c r="D21" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="E21" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="F21" s="14">
-        <v>5015</v>
-      </c>
-      <c r="G21" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="H21" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="34" t="s">
-        <v>111</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" s="19" t="s">
-        <v>112</v>
-      </c>
-      <c r="F22" s="14">
-        <v>5209</v>
-      </c>
-      <c r="G22" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H22" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B23" s="34" t="s">
-        <v>113</v>
-      </c>
-      <c r="C23" s="31" t="s">
-        <v>19</v>
-      </c>
-      <c r="D23" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="E23" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="F23" s="14">
-        <v>5370</v>
-      </c>
-      <c r="G23" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H23" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B24" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="C24" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="E24" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="F24" s="14">
-        <v>5405</v>
-      </c>
-      <c r="G24" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H24" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B25" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="C25" s="31" t="s">
-        <v>19</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="E25" s="19" t="s">
-        <v>117</v>
-      </c>
-      <c r="F25" s="14">
-        <v>6530</v>
-      </c>
-      <c r="G25" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H25" s="22" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B26" s="34" t="s">
-        <v>118</v>
-      </c>
-      <c r="C26" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="D26" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="E26" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="F26" s="14">
-        <v>7800</v>
-      </c>
-      <c r="G26" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H26" s="22" t="s">
-        <v>81</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2294,20 +1693,6 @@
     <hyperlink ref="H10" r:id="rId5"/>
     <hyperlink ref="H11" r:id="rId6"/>
     <hyperlink ref="H12" r:id="rId7"/>
-    <hyperlink ref="H13" r:id="rId8"/>
-    <hyperlink ref="H14" r:id="rId9"/>
-    <hyperlink ref="H15" r:id="rId10"/>
-    <hyperlink ref="H16" r:id="rId11"/>
-    <hyperlink ref="H17" r:id="rId12"/>
-    <hyperlink ref="H18" r:id="rId13"/>
-    <hyperlink ref="H19" r:id="rId14"/>
-    <hyperlink ref="H20" r:id="rId15"/>
-    <hyperlink ref="H21" r:id="rId16"/>
-    <hyperlink ref="H22" r:id="rId17"/>
-    <hyperlink ref="H23" r:id="rId18"/>
-    <hyperlink ref="H24" r:id="rId19"/>
-    <hyperlink ref="H25" r:id="rId20"/>
-    <hyperlink ref="H26" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2316,7 +1701,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H14"/>
+  <dimension ref="B2:H8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -2331,7 +1716,7 @@
   <sheetData>
     <row r="2" ht="34" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>120</v>
+        <v>78</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -2342,7 +1727,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
@@ -2353,10 +1738,10 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="26" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="D5" s="26" t="s">
         <v>8</v>
@@ -2365,220 +1750,82 @@
         <v>28</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>123</v>
+        <v>81</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>124</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="34" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="D6" s="34" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="F6" s="30">
-        <v>3119</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="H6" s="35" t="s">
-        <v>128</v>
+        <v>85</v>
+      </c>
+      <c r="F6" s="35">
+        <v>2600</v>
+      </c>
+      <c r="G6" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="H6" s="37" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="34" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="F7" s="30">
-        <v>2140</v>
-      </c>
-      <c r="G7" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="H7" s="35" t="s">
-        <v>128</v>
+        <v>88</v>
+      </c>
+      <c r="F7" s="35">
+        <v>2632</v>
+      </c>
+      <c r="G7" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="H7" s="37" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="34" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>126</v>
+        <v>84</v>
       </c>
       <c r="D8" s="34" t="s">
         <v>23</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="F8" s="30">
-        <v>2375</v>
+        <v>5900</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="H8" s="35" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="D9" s="34" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="F9" s="36">
-        <v>6095.4</v>
-      </c>
-      <c r="G9" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="H9" s="35" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="D10" s="34" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="F10" s="36">
-        <v>999</v>
-      </c>
-      <c r="G10" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="H10" s="35" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="D11" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="F11" s="36">
-        <v>7509</v>
-      </c>
-      <c r="G11" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="H11" s="35" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B12" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D12" s="34" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="F12" s="30">
-        <v>4425</v>
-      </c>
-      <c r="G12" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="H12" s="35" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B13" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D13" s="34" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="F13" s="30">
-        <v>5015</v>
-      </c>
-      <c r="G13" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="H13" s="35" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B14" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="D14" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="19" t="s">
-        <v>100</v>
-      </c>
-      <c r="F14" s="30">
-        <v>2600</v>
-      </c>
-      <c r="G14" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="H14" s="35" t="s">
-        <v>128</v>
+        <v>90</v>
+      </c>
+      <c r="H8" s="37" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -2593,7 +1840,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H8"/>
+  <dimension ref="B2:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -2607,7 +1854,7 @@
   <sheetData>
     <row r="2" ht="34" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="38" t="s">
-        <v>138</v>
+        <v>92</v>
       </c>
       <c r="C2" s="38"/>
       <c r="D2" s="38"/>
@@ -2618,7 +1865,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
-        <v>139</v>
+        <v>93</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
@@ -2629,94 +1876,71 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="26" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>140</v>
+        <v>94</v>
       </c>
       <c r="D5" s="26" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>141</v>
+        <v>95</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>142</v>
+        <v>96</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>143</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="34" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="C6" s="39" t="s">
-        <v>144</v>
+        <v>98</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>129</v>
+        <v>84</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>130</v>
+        <v>85</v>
       </c>
       <c r="G6" s="40" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
       <c r="H6" s="41" t="s">
-        <v>132</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="34" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="C7" s="39" t="s">
-        <v>144</v>
+        <v>98</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>129</v>
+        <v>84</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>133</v>
+        <v>88</v>
       </c>
       <c r="G7" s="40" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
       <c r="H7" s="41" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="34" t="s">
-        <v>125</v>
-      </c>
-      <c r="C8" s="39" t="s">
-        <v>144</v>
-      </c>
-      <c r="D8" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>129</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="G8" s="40" t="s">
-        <v>145</v>
-      </c>
-      <c r="H8" s="41" t="s">
-        <v>136</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feat: Consolidar canasta mensual completa y reporte Excel de 5 hojas
</commit_message>
<xml_diff>
--- a/reporte_supermercados.xlsx
+++ b/reporte_supermercados.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="172">
   <si>
     <t>🛒 REPORTE RPA: COMPARADOR DE PRECIOS Y CANASTA INTELIGENTE</t>
   </si>
@@ -35,49 +35,58 @@
     <t>💸 AHORRO MÁXIMO</t>
   </si>
   <si>
+    <t>Día %</t>
+  </si>
+  <si>
+    <t>📊 EVALUACIÓN COMPARATIVA: COSTO TOTAL DE LA CANASTA COMPLETA</t>
+  </si>
+  <si>
+    <t>Supermercado</t>
+  </si>
+  <si>
+    <t>Costo Canasta Total</t>
+  </si>
+  <si>
+    <t>Artículos Disponibles</t>
+  </si>
+  <si>
+    <t>Artículos con Problema</t>
+  </si>
+  <si>
+    <t>Precios Más Bajos Ganados</t>
+  </si>
+  <si>
+    <t>Diferencia vs Mejor</t>
+  </si>
+  <si>
+    <t>Estado / Recomendación</t>
+  </si>
+  <si>
+    <t>Carrefour</t>
+  </si>
+  <si>
+    <t>9 de 9</t>
+  </si>
+  <si>
+    <t>1 productos</t>
+  </si>
+  <si>
+    <t>+$6.430,70</t>
+  </si>
+  <si>
+    <t>Más costoso</t>
+  </si>
+  <si>
     <t>COTO</t>
   </si>
   <si>
-    <t>📊 EVALUACIÓN COMPARATIVA: COSTO TOTAL DE LA CANASTA COMPLETA</t>
-  </si>
-  <si>
-    <t>Supermercado</t>
-  </si>
-  <si>
-    <t>Costo Canasta Total</t>
-  </si>
-  <si>
-    <t>Artículos Disponibles</t>
-  </si>
-  <si>
-    <t>Artículos con Problema</t>
-  </si>
-  <si>
-    <t>Precios Más Bajos Ganados</t>
-  </si>
-  <si>
-    <t>Diferencia vs Mejor</t>
-  </si>
-  <si>
-    <t>Estado / Recomendación</t>
-  </si>
-  <si>
-    <t>Carrefour</t>
-  </si>
-  <si>
-    <t>2 de 2</t>
-  </si>
-  <si>
-    <t>0 productos</t>
-  </si>
-  <si>
-    <t>+$31,00</t>
-  </si>
-  <si>
-    <t>Más costoso</t>
-  </si>
-  <si>
-    <t>1 productos</t>
+    <t>3 productos</t>
+  </si>
+  <si>
+    <t>+$23.531,69</t>
+  </si>
+  <si>
+    <t>5 productos</t>
   </si>
   <si>
     <t>Mejor opción</t>
@@ -86,12 +95,6 @@
     <t>🏆 RECOMENDADO</t>
   </si>
   <si>
-    <t>Día %</t>
-  </si>
-  <si>
-    <t>+$739,50</t>
-  </si>
-  <si>
     <t>🛒 PRODUCTO GANADOR POR ARTÍCULO (MEJOR PRECIO)</t>
   </si>
   <si>
@@ -149,9 +152,96 @@
     <t>-$510,5</t>
   </si>
   <si>
+    <t>FIDEOS</t>
+  </si>
+  <si>
+    <t>Fideos Tirabuzon N28 Matarazzo 500 Gr.</t>
+  </si>
+  <si>
+    <t>COTO ($1.750)</t>
+  </si>
+  <si>
+    <t>-$510</t>
+  </si>
+  <si>
+    <t>ACEITE</t>
+  </si>
+  <si>
+    <t>Aceite de Girasol Dia 1,5 Lt.</t>
+  </si>
+  <si>
+    <t>COTO ($6.530)</t>
+  </si>
+  <si>
+    <t>-$1.930</t>
+  </si>
+  <si>
+    <t>YERBA</t>
+  </si>
+  <si>
+    <t>Yerba Mate Mañanita 4 Flex 1 Kg.</t>
+  </si>
+  <si>
+    <t>COTO ($5.370)</t>
+  </si>
+  <si>
+    <t>-$1.580</t>
+  </si>
+  <si>
+    <t>AZUCAR</t>
+  </si>
+  <si>
+    <t>🏆 Carrefour</t>
+  </si>
+  <si>
+    <t>Azúcar común Azucel tipo A bolsa 1 kg.</t>
+  </si>
+  <si>
+    <t>COTO ($1.567)</t>
+  </si>
+  <si>
+    <t>-$177</t>
+  </si>
+  <si>
+    <t>CAFE</t>
+  </si>
+  <si>
+    <t>Cafe Instantáneo Nescafe Dolca Mixes Caramel Doypack X 125 Gr.</t>
+  </si>
+  <si>
+    <t>COTO ($29.671)</t>
+  </si>
+  <si>
+    <t>-$26.096,2</t>
+  </si>
+  <si>
+    <t>GALLETITAS</t>
+  </si>
+  <si>
+    <t>Galletitas Dulces Pepas Con Membrillo 9 De Oro 140g</t>
+  </si>
+  <si>
+    <t>Día % ($6.649)</t>
+  </si>
+  <si>
+    <t>-$5.379</t>
+  </si>
+  <si>
+    <t>PAPEL HIGIENICO</t>
+  </si>
+  <si>
+    <t>Papel Higiénico CAMPANITA Soft Simple Hoja Paquete 4 Unidades</t>
+  </si>
+  <si>
+    <t>Carrefour ($4.250)</t>
+  </si>
+  <si>
+    <t>-$1.903,01</t>
+  </si>
+  <si>
     <t xml:space="preserve">💡 CONCLUSIÓN Y ESTRATEGIA RECOMENDADA POR EL BOT RPA:
-1. Si realizás toda la compra mensual en un único lugar: El supermercado más conveniente es COTO con un costo de $4.249,00.
-2. Si realizás una compra combinada (comprando cada producto en su supermercado ganador): Pagás solo $3.738,50, ahorrando un total de $1.250,00.
+1. Si realizás toda la compra mensual en un único lugar: El supermercado más conveniente es Día % con un costo de $29.222,30.
+2. Si realizás una compra combinada (comprando cada producto en su supermercado ganador): Pagás solo $21.950,29, ahorrando un total de $30.803,70.
 3. Podés verificar el detalle de stock y sustituciones rechazadas en la pestaña "⚠️ Disponibilidad y Stock".</t>
   </si>
   <si>
@@ -176,12 +266,33 @@
     <t>-$510,50</t>
   </si>
   <si>
+    <t>-$510,00</t>
+  </si>
+  <si>
+    <t>-$1.930,00</t>
+  </si>
+  <si>
+    <t>-$1.580,00</t>
+  </si>
+  <si>
+    <t>-$177,00</t>
+  </si>
+  <si>
+    <t>-$26.096,20</t>
+  </si>
+  <si>
+    <t>-$5.379,00</t>
+  </si>
+  <si>
     <t>TOTAL CANASTA</t>
   </si>
   <si>
     <t>Óptima Combinada</t>
   </si>
   <si>
+    <t>-$30.803,70</t>
+  </si>
+  <si>
     <t>📊 RANKING GENERAL: TODOS LOS PRODUCTOS DE MENOR A MAYOR PRECIO</t>
   </si>
   <si>
@@ -218,31 +329,112 @@
     <t>🥈 2° Puesto</t>
   </si>
   <si>
+    <t>🥉 3° Puesto</t>
+  </si>
+  <si>
+    <t>#4</t>
+  </si>
+  <si>
+    <t>Azucar Ledesma Refinado Superior 1 Kg.</t>
+  </si>
+  <si>
+    <t>#5</t>
+  </si>
+  <si>
+    <t>#6</t>
+  </si>
+  <si>
+    <t>Azúcar Superior Real LEDESMA 1kg</t>
+  </si>
+  <si>
+    <t>#7</t>
+  </si>
+  <si>
+    <t>Fideos tallarin N5 Lucchetti 500 g.</t>
+  </si>
+  <si>
+    <t>#8</t>
+  </si>
+  <si>
+    <t>Fideos Spaghetti N° 7 LUCCHETTI 500g</t>
+  </si>
+  <si>
+    <t>#9</t>
+  </si>
+  <si>
     <t>Arroz largo fino Molinos Ala 1 kg.</t>
   </si>
   <si>
-    <t>🥉 3° Puesto</t>
+    <t>#10</t>
   </si>
   <si>
     <t>Arroz Largo Fino LUCCHETTI 1kg</t>
   </si>
   <si>
-    <t>#4</t>
-  </si>
-  <si>
-    <t>#5</t>
+    <t>#11</t>
+  </si>
+  <si>
+    <t>#12</t>
   </si>
   <si>
     <t>Leche Protein La Serenisima 1L</t>
   </si>
   <si>
-    <t>#6</t>
+    <t>#13</t>
+  </si>
+  <si>
+    <t>#14</t>
+  </si>
+  <si>
+    <t>Papel Higiénico Doble Hoja 30mts 6 Ud.</t>
+  </si>
+  <si>
+    <t>#15</t>
+  </si>
+  <si>
+    <t>Galletitas clásicas Traviata x5 108 g</t>
+  </si>
+  <si>
+    <t>#16</t>
   </si>
   <si>
     <t>Danette Postre Sabor Dulce De Leche Pack X2 95 Gr.</t>
   </si>
   <si>
-    <t>#7</t>
+    <t>#17</t>
+  </si>
+  <si>
+    <t>#18</t>
+  </si>
+  <si>
+    <t>#19</t>
+  </si>
+  <si>
+    <t>Papel higiénico doble hoja Higienol plus x4 30 mts</t>
+  </si>
+  <si>
+    <t>#20</t>
+  </si>
+  <si>
+    <t>#21</t>
+  </si>
+  <si>
+    <t>Yerba mate Playadito suave con palo 1 kg.</t>
+  </si>
+  <si>
+    <t>#22</t>
+  </si>
+  <si>
+    <t>Yerba Mate 4 Flex Mañanita Paq 1 Kgm</t>
+  </si>
+  <si>
+    <t>#23</t>
+  </si>
+  <si>
+    <t>Aceite de girasol alto omega Carrefour Classic pet 1.5 lts</t>
+  </si>
+  <si>
+    <t>#24</t>
   </si>
   <si>
     <t>COCA COLA, 2.25L</t>
@@ -252,6 +444,30 @@
   </si>
   <si>
     <t>🔎 Individual</t>
+  </si>
+  <si>
+    <t>#25</t>
+  </si>
+  <si>
+    <t>Aceite Girasol CAÑUELAS Botella 1.5 L</t>
+  </si>
+  <si>
+    <t>#26</t>
+  </si>
+  <si>
+    <t>Galletitas Oreo Rellenas con Crema Sabor Original 354 Gr.</t>
+  </si>
+  <si>
+    <t>#27</t>
+  </si>
+  <si>
+    <t>Nescafé Dolca Suave 170 grs</t>
+  </si>
+  <si>
+    <t>#28</t>
+  </si>
+  <si>
+    <t>Cafe Tostado Molido Super Cabrales 500 Grm</t>
   </si>
   <si>
     <t>🔎 HISTORIAL DE BÚSQUEDAS INDIVIDUALES Y VALIDACIONES EN VIVO</t>
@@ -1011,7 +1227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H22"/>
+  <dimension ref="B2:H29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1068,15 +1284,15 @@
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="5">
-        <v>4249</v>
+        <v>29222.3</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="6">
-        <v>3738.5</v>
+        <v>21950.29</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6">
-        <v>1250</v>
+        <v>30803.699999999997</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
@@ -1118,7 +1334,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="10">
-        <v>4280</v>
+        <v>35653</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>16</v>
@@ -1138,10 +1354,10 @@
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="14">
-        <v>4249</v>
+        <v>20</v>
+      </c>
+      <c r="C11" s="10">
+        <v>52753.99</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>16</v>
@@ -1150,21 +1366,21 @@
         <v>0</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="16" t="s">
+      <c r="G11" s="12" t="s">
         <v>22</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="10">
-        <v>4988.5</v>
+        <v>6</v>
+      </c>
+      <c r="C12" s="14">
+        <v>29222.3</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>16</v>
@@ -1173,18 +1389,18 @@
         <v>0</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="H12" s="13" t="s">
-        <v>19</v>
+      <c r="H12" s="16" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
@@ -1195,110 +1411,271 @@
     </row>
     <row r="15" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E16" s="14">
         <v>2250</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H16" s="22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E17" s="14">
         <v>1488.5</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H17" s="22" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B19" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="23"/>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="23"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" s="14">
+        <v>1240</v>
+      </c>
+      <c r="F18" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="G18" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="H18" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="14">
+        <v>4600</v>
+      </c>
+      <c r="F19" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="G19" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="H19" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="14">
+        <v>3790</v>
+      </c>
+      <c r="F20" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="G20" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="E21" s="14">
+        <v>1390</v>
+      </c>
+      <c r="F21" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H21" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="E22" s="14">
+        <v>3574.8</v>
+      </c>
+      <c r="F22" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="H22" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B23" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="14">
+        <v>1270</v>
+      </c>
+      <c r="F23" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="G23" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="H23" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="E24" s="14">
+        <v>2346.99</v>
+      </c>
+      <c r="F24" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="G24" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="H24" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" s="23"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1312,11 +1689,18 @@
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="B8:H8"/>
     <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B19:H22"/>
+    <mergeCell ref="B26:H29"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H16" r:id="rId1"/>
     <hyperlink ref="H17" r:id="rId2"/>
+    <hyperlink ref="H18" r:id="rId3"/>
+    <hyperlink ref="H19" r:id="rId4"/>
+    <hyperlink ref="H20" r:id="rId5"/>
+    <hyperlink ref="H21" r:id="rId6"/>
+    <hyperlink ref="H22" r:id="rId7"/>
+    <hyperlink ref="H23" r:id="rId8"/>
+    <hyperlink ref="H24" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1325,7 +1709,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H8"/>
+  <dimension ref="B2:H15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1337,7 +1721,7 @@
   <sheetData>
     <row r="2" ht="34" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -1348,7 +1732,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
-        <v>46</v>
+        <v>76</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
@@ -1359,30 +1743,30 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="26" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C5" s="26" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="26" t="s">
-        <v>23</v>
-      </c>
       <c r="F5" s="26" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>49</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="27">
         <v>2340</v>
@@ -1394,18 +1778,18 @@
         <v>3500</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="28">
         <v>2250</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" s="27">
         <v>1940</v>
@@ -1417,36 +1801,197 @@
         <v>1488.5</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G7" s="28">
         <v>1488.5</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="30">
-        <v>4280</v>
-      </c>
-      <c r="D8" s="14">
-        <v>4249</v>
-      </c>
-      <c r="E8" s="30">
-        <v>4988.5</v>
-      </c>
-      <c r="F8" s="15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="27">
+        <v>1749</v>
+      </c>
+      <c r="D8" s="27">
+        <v>1750</v>
+      </c>
+      <c r="E8" s="14">
+        <v>1240</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="28">
+        <v>1240</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="27">
+        <v>5405</v>
+      </c>
+      <c r="D9" s="27">
+        <v>6530</v>
+      </c>
+      <c r="E9" s="14">
+        <v>4600</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="28">
+        <v>4600</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="G8" s="14">
-        <v>3738.5</v>
-      </c>
-      <c r="H8" s="15" t="s">
-        <v>50</v>
+      <c r="C10" s="27">
+        <v>5209</v>
+      </c>
+      <c r="D10" s="27">
+        <v>5370</v>
+      </c>
+      <c r="E10" s="14">
+        <v>3790</v>
+      </c>
+      <c r="F10" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="28">
+        <v>3790</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="14">
+        <v>1390</v>
+      </c>
+      <c r="D11" s="27">
+        <v>1567</v>
+      </c>
+      <c r="E11" s="27">
+        <v>1470</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="28">
+        <v>1390</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="27">
+        <v>10210</v>
+      </c>
+      <c r="D12" s="27">
+        <v>29671</v>
+      </c>
+      <c r="E12" s="14">
+        <v>3574.8</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="28">
+        <v>3574.8</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="27">
+        <v>3160</v>
+      </c>
+      <c r="D13" s="14">
+        <v>1270</v>
+      </c>
+      <c r="E13" s="27">
+        <v>6649</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="28">
+        <v>1270</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="27">
+        <v>4250</v>
+      </c>
+      <c r="D14" s="14">
+        <v>2346.99</v>
+      </c>
+      <c r="E14" s="27">
+        <v>2910</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14" s="28">
+        <v>2346.99</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="C15" s="30">
+        <v>35653</v>
+      </c>
+      <c r="D15" s="30">
+        <v>52753.99</v>
+      </c>
+      <c r="E15" s="14">
+        <v>29222.3</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" s="14">
+        <v>21950.29</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1461,7 +2006,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H12"/>
+  <dimension ref="B2:H33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1476,7 +2021,7 @@
   <sheetData>
     <row r="2" ht="34" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -1487,7 +2032,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
@@ -1498,186 +2043,669 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="26" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="C5" s="26" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="26" t="s">
-        <v>57</v>
+        <v>94</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>59</v>
+        <v>96</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>60</v>
+        <v>97</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>61</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="16" t="s">
-        <v>62</v>
+        <v>99</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F6" s="28">
-        <v>1488.5</v>
+        <v>1240</v>
       </c>
       <c r="G6" s="32" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="33" t="s">
-        <v>65</v>
+        <v>102</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F7" s="28">
-        <v>1940</v>
+        <v>1270</v>
       </c>
       <c r="G7" s="32" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="H7" s="22" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="33" t="s">
-        <v>67</v>
+        <v>103</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="F8" s="28">
-        <v>1999</v>
+        <v>1390</v>
       </c>
       <c r="G8" s="32" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="34" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="F9" s="10">
-        <v>2250</v>
+        <v>1470</v>
       </c>
       <c r="G9" s="32" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="34" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="F10" s="10">
-        <v>2340</v>
+        <v>1488.5</v>
       </c>
       <c r="G10" s="32" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="34" t="s">
-        <v>72</v>
+        <v>107</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="E11" s="19" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="F11" s="10">
-        <v>3500</v>
+        <v>1567</v>
       </c>
       <c r="G11" s="32" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="H11" s="22" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="34" t="s">
-        <v>74</v>
+        <v>109</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>76</v>
+        <v>110</v>
       </c>
       <c r="F12" s="10">
+        <v>1749</v>
+      </c>
+      <c r="G12" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H12" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="34" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="F13" s="10">
+        <v>1750</v>
+      </c>
+      <c r="G13" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H13" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="19" t="s">
+        <v>114</v>
+      </c>
+      <c r="F14" s="10">
+        <v>1940</v>
+      </c>
+      <c r="G14" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H14" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="F15" s="10">
+        <v>1999</v>
+      </c>
+      <c r="G15" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H15" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="C16" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" s="10">
+        <v>2250</v>
+      </c>
+      <c r="G16" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H16" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="F17" s="10">
+        <v>2340</v>
+      </c>
+      <c r="G17" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H17" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" s="10">
+        <v>2346.99</v>
+      </c>
+      <c r="G18" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H18" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="34" t="s">
+        <v>121</v>
+      </c>
+      <c r="C19" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="F19" s="10">
+        <v>2910</v>
+      </c>
+      <c r="G19" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H19" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="C20" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E20" s="19" t="s">
+        <v>124</v>
+      </c>
+      <c r="F20" s="10">
+        <v>3160</v>
+      </c>
+      <c r="G20" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="C21" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="F21" s="10">
+        <v>3500</v>
+      </c>
+      <c r="G21" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H21" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="34" t="s">
+        <v>127</v>
+      </c>
+      <c r="C22" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="F22" s="10">
+        <v>3574.8</v>
+      </c>
+      <c r="G22" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H22" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B23" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="C23" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="F23" s="10">
+        <v>3790</v>
+      </c>
+      <c r="G23" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H23" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="34" t="s">
+        <v>129</v>
+      </c>
+      <c r="C24" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="F24" s="10">
+        <v>4250</v>
+      </c>
+      <c r="G24" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H24" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="34" t="s">
+        <v>131</v>
+      </c>
+      <c r="C25" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="F25" s="10">
+        <v>4600</v>
+      </c>
+      <c r="G25" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H25" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="34" t="s">
+        <v>132</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E26" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="F26" s="10">
+        <v>5209</v>
+      </c>
+      <c r="G26" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H26" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B27" s="34" t="s">
+        <v>134</v>
+      </c>
+      <c r="C27" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="E27" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="F27" s="10">
+        <v>5370</v>
+      </c>
+      <c r="G27" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H27" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B28" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" s="10">
+        <v>5405</v>
+      </c>
+      <c r="G28" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H28" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B29" s="34" t="s">
+        <v>138</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="F29" s="10">
         <v>5900</v>
       </c>
-      <c r="G12" s="32" t="s">
-        <v>77</v>
-      </c>
-      <c r="H12" s="22" t="s">
-        <v>64</v>
+      <c r="G29" s="32" t="s">
+        <v>141</v>
+      </c>
+      <c r="H29" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B30" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="C30" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="E30" s="19" t="s">
+        <v>143</v>
+      </c>
+      <c r="F30" s="10">
+        <v>6530</v>
+      </c>
+      <c r="G30" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H30" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B31" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="C31" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="F31" s="10">
+        <v>6649</v>
+      </c>
+      <c r="G31" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H31" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B32" s="34" t="s">
+        <v>146</v>
+      </c>
+      <c r="C32" s="31" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="E32" s="19" t="s">
+        <v>147</v>
+      </c>
+      <c r="F32" s="10">
+        <v>10210</v>
+      </c>
+      <c r="G32" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H32" s="22" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B33" s="34" t="s">
+        <v>148</v>
+      </c>
+      <c r="C33" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="E33" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="F33" s="10">
+        <v>29671</v>
+      </c>
+      <c r="G33" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H33" s="22" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1693,6 +2721,27 @@
     <hyperlink ref="H10" r:id="rId5"/>
     <hyperlink ref="H11" r:id="rId6"/>
     <hyperlink ref="H12" r:id="rId7"/>
+    <hyperlink ref="H13" r:id="rId8"/>
+    <hyperlink ref="H14" r:id="rId9"/>
+    <hyperlink ref="H15" r:id="rId10"/>
+    <hyperlink ref="H16" r:id="rId11"/>
+    <hyperlink ref="H17" r:id="rId12"/>
+    <hyperlink ref="H18" r:id="rId13"/>
+    <hyperlink ref="H19" r:id="rId14"/>
+    <hyperlink ref="H20" r:id="rId15"/>
+    <hyperlink ref="H21" r:id="rId16"/>
+    <hyperlink ref="H22" r:id="rId17"/>
+    <hyperlink ref="H23" r:id="rId18"/>
+    <hyperlink ref="H24" r:id="rId19"/>
+    <hyperlink ref="H25" r:id="rId20"/>
+    <hyperlink ref="H26" r:id="rId21"/>
+    <hyperlink ref="H27" r:id="rId22"/>
+    <hyperlink ref="H28" r:id="rId23"/>
+    <hyperlink ref="H29" r:id="rId24"/>
+    <hyperlink ref="H30" r:id="rId25"/>
+    <hyperlink ref="H31" r:id="rId26"/>
+    <hyperlink ref="H32" r:id="rId27"/>
+    <hyperlink ref="H33" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1716,7 +2765,7 @@
   <sheetData>
     <row r="2" ht="34" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="24" t="s">
-        <v>78</v>
+        <v>150</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
@@ -1727,7 +2776,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
-        <v>79</v>
+        <v>151</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
@@ -1738,94 +2787,94 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="26" t="s">
-        <v>80</v>
+        <v>152</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>57</v>
+        <v>94</v>
       </c>
       <c r="D5" s="26" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>59</v>
+        <v>96</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>81</v>
+        <v>153</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>82</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="34" t="s">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>84</v>
+        <v>156</v>
       </c>
       <c r="D6" s="34" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>85</v>
+        <v>157</v>
       </c>
       <c r="F6" s="35">
         <v>2600</v>
       </c>
       <c r="G6" s="36" t="s">
-        <v>86</v>
+        <v>158</v>
       </c>
       <c r="H6" s="37" t="s">
-        <v>87</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="34" t="s">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>84</v>
+        <v>156</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E7" s="19" t="s">
-        <v>88</v>
+        <v>160</v>
       </c>
       <c r="F7" s="35">
         <v>2632</v>
       </c>
       <c r="G7" s="36" t="s">
-        <v>86</v>
+        <v>158</v>
       </c>
       <c r="H7" s="37" t="s">
-        <v>89</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="34" t="s">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>84</v>
+        <v>156</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="E8" s="19" t="s">
-        <v>76</v>
+        <v>140</v>
       </c>
       <c r="F8" s="30">
         <v>5900</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>90</v>
+        <v>162</v>
       </c>
       <c r="H8" s="37" t="s">
-        <v>91</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -1854,7 +2903,7 @@
   <sheetData>
     <row r="2" ht="34" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="38" t="s">
-        <v>92</v>
+        <v>164</v>
       </c>
       <c r="C2" s="38"/>
       <c r="D2" s="38"/>
@@ -1865,7 +2914,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="25" t="s">
-        <v>93</v>
+        <v>165</v>
       </c>
       <c r="C3" s="25"/>
       <c r="D3" s="25"/>
@@ -1876,71 +2925,71 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="26" t="s">
-        <v>80</v>
+        <v>152</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>94</v>
+        <v>166</v>
       </c>
       <c r="D5" s="26" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>57</v>
+        <v>94</v>
       </c>
       <c r="F5" s="26" t="s">
-        <v>95</v>
+        <v>167</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>96</v>
+        <v>168</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>97</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="34" t="s">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="C6" s="39" t="s">
-        <v>98</v>
+        <v>170</v>
       </c>
       <c r="D6" s="31" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>84</v>
+        <v>156</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>85</v>
+        <v>157</v>
       </c>
       <c r="G6" s="40" t="s">
-        <v>99</v>
+        <v>171</v>
       </c>
       <c r="H6" s="41" t="s">
-        <v>87</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="34" t="s">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="C7" s="39" t="s">
-        <v>98</v>
+        <v>170</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>84</v>
+        <v>156</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>88</v>
+        <v>160</v>
       </c>
       <c r="G7" s="40" t="s">
-        <v>99</v>
+        <v>171</v>
       </c>
       <c r="H7" s="41" t="s">
-        <v>89</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>